<commit_message>
Fix breakdown year filter, remove favicon, fix duplicate keys, update quotation template
- Fix strftime %% escaping bug in breakdown filter query (no params = no unescaping)
- Remove favicon with empty data URI
- Fix duplicate React keys in abattoir dropdowns (NewQuote, STTTrainingReport)
- Change quotation template discount text color to red
- Update vite proxy to port 8001

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Quotation Template.xlsx
+++ b/Quotation Template.xlsx
@@ -25,7 +25,7 @@
     <numFmt numFmtId="168" formatCode="0\ &quot;km&quot;"/>
     <numFmt numFmtId="169" formatCode="_-&quot;£&quot;* #,##0.00_-;\-&quot;£&quot;* #,##0.00_-;_-&quot;£&quot;* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="30">
+  <fonts count="31">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -244,6 +244,12 @@
       <color rgb="FF0070C0"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FFFF0000"/>
+      <sz val="10"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -990,7 +996,7 @@
     </xf>
     <xf numFmtId="169" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="242">
+  <cellXfs count="243">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1649,6 +1655,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="34" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="23" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="22" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="30" fillId="0" borderId="50" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2770,7 +2779,7 @@
       <c r="K33" s="85" t="n"/>
     </row>
     <row r="34" ht="16.5" customFormat="1" customHeight="1" s="218">
-      <c r="A34" s="219" t="inlineStr">
+      <c r="A34" s="242" t="inlineStr">
         <is>
           <t>Conducting an audit verification &amp; sampling enables us to provide you with a discount.</t>
         </is>
@@ -2977,8 +2986,8 @@
     <mergeCell ref="H41:I41"/>
     <mergeCell ref="A27:I27"/>
     <mergeCell ref="A3:C3"/>
+    <mergeCell ref="D36:E36"/>
     <mergeCell ref="A12:C12"/>
-    <mergeCell ref="D36:E36"/>
     <mergeCell ref="D16:I16"/>
     <mergeCell ref="D7:I7"/>
     <mergeCell ref="A2:C2"/>

</xml_diff>

<commit_message>
Fix quotation discount formula to subtract instead of add
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Quotation Template.xlsx
+++ b/Quotation Template.xlsx
@@ -2902,7 +2902,7 @@
       <c r="G39" s="180" t="n"/>
       <c r="H39" s="236" t="n"/>
       <c r="I39" s="237">
-        <f>I31-I38</f>
+        <f>I31+I38</f>
         <v/>
       </c>
     </row>
@@ -2986,9 +2986,9 @@
     <mergeCell ref="H41:I41"/>
     <mergeCell ref="A27:I27"/>
     <mergeCell ref="A3:C3"/>
-    <mergeCell ref="D36:E36"/>
     <mergeCell ref="A12:C12"/>
     <mergeCell ref="D16:I16"/>
+    <mergeCell ref="D36:E36"/>
     <mergeCell ref="D7:I7"/>
     <mergeCell ref="A2:C2"/>
     <mergeCell ref="B28:D28"/>

</xml_diff>

<commit_message>
Add R currency format to Skills Programme amount column in quotation template
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Quotation Template.xlsx
+++ b/Quotation Template.xlsx
@@ -2573,7 +2573,7 @@
       </c>
       <c r="B22" s="72" t="n"/>
       <c r="C22" s="78" t="n"/>
-      <c r="D22" s="77" t="n"/>
+      <c r="D22" s="186" t="n"/>
       <c r="E22" s="78" t="n"/>
       <c r="F22" s="186" t="n"/>
       <c r="G22" s="187" t="n"/>
@@ -2591,7 +2591,7 @@
       </c>
       <c r="B23" s="72" t="n"/>
       <c r="C23" s="78" t="n"/>
-      <c r="D23" s="79" t="n"/>
+      <c r="D23" s="186" t="n"/>
       <c r="E23" s="78" t="n"/>
       <c r="F23" s="186" t="n"/>
       <c r="G23" s="187" t="n"/>
@@ -2609,7 +2609,7 @@
       </c>
       <c r="B24" s="72" t="n"/>
       <c r="C24" s="78" t="n"/>
-      <c r="D24" s="79" t="n"/>
+      <c r="D24" s="186" t="n"/>
       <c r="E24" s="78" t="n"/>
       <c r="F24" s="186" t="n"/>
       <c r="G24" s="187" t="n"/>
@@ -2627,7 +2627,7 @@
       </c>
       <c r="B25" s="72" t="n"/>
       <c r="C25" s="78" t="n"/>
-      <c r="D25" s="79" t="n"/>
+      <c r="D25" s="186" t="n"/>
       <c r="E25" s="78" t="n"/>
       <c r="F25" s="186" t="n"/>
       <c r="G25" s="187" t="n"/>
@@ -2645,7 +2645,7 @@
       </c>
       <c r="B26" s="109" t="n"/>
       <c r="C26" s="80" t="n"/>
-      <c r="D26" s="81" t="n"/>
+      <c r="D26" s="190" t="n"/>
       <c r="E26" s="80" t="n"/>
       <c r="F26" s="190" t="n"/>
       <c r="G26" s="191" t="n"/>

</xml_diff>

<commit_message>
Fix quotation TOTAL formula to include Skills Programme amount (column D)
The TOTAL column was only summing Slaughter + Distance + Accommodation,
missing the Skills Programme amount entirely.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Quotation Template.xlsx
+++ b/Quotation Template.xlsx
@@ -2579,7 +2579,7 @@
       <c r="G22" s="187" t="n"/>
       <c r="H22" s="188" t="n"/>
       <c r="I22" s="186">
-        <f>SUM(F22+(G22*5.5)+H22)</f>
+        <f>SUM(D22+F22+(G22*5.5)+H22)</f>
         <v/>
       </c>
       <c r="J22" s="189" t="n"/>
@@ -2597,7 +2597,7 @@
       <c r="G23" s="187" t="n"/>
       <c r="H23" s="188" t="n"/>
       <c r="I23" s="186">
-        <f>SUM(F23+(G23*5.5)+H23)</f>
+        <f>SUM(D23+F23+(G23*5.5)+H23)</f>
         <v/>
       </c>
       <c r="J23" s="189" t="n"/>
@@ -2615,7 +2615,7 @@
       <c r="G24" s="187" t="n"/>
       <c r="H24" s="188" t="n"/>
       <c r="I24" s="186">
-        <f>SUM(F24+(G24*5.5)+H24)</f>
+        <f>SUM(D24+F24+(G24*5.5)+H24)</f>
         <v/>
       </c>
       <c r="J24" s="189" t="n"/>
@@ -2633,7 +2633,7 @@
       <c r="G25" s="187" t="n"/>
       <c r="H25" s="188" t="n"/>
       <c r="I25" s="186">
-        <f>SUM(F25+(G25*5.5)+H25)</f>
+        <f>SUM(D25+F25+(G25*5.5)+H25)</f>
         <v/>
       </c>
       <c r="J25" s="189" t="n"/>
@@ -2651,7 +2651,7 @@
       <c r="G26" s="191" t="n"/>
       <c r="H26" s="192" t="n"/>
       <c r="I26" s="190">
-        <f>SUM(F26+(G26*5.5)+H26)</f>
+        <f>SUM(D26+F26+(G26*5.5)+H26)</f>
         <v/>
       </c>
       <c r="J26" s="189" t="n"/>
@@ -2796,7 +2796,7 @@
       <c r="G34" s="222" t="n"/>
       <c r="H34" s="223" t="n"/>
       <c r="I34" s="224">
-        <f>SUM(F34+(G34*5.5)+H34)</f>
+        <f>SUM(D34+F34+(G34*5.5)+H34)</f>
         <v/>
       </c>
       <c r="J34" s="189" t="n"/>
@@ -2831,7 +2831,7 @@
       <c r="G35" s="227" t="n"/>
       <c r="H35" s="226" t="n"/>
       <c r="I35" s="228">
-        <f>SUM(F35+(G35*5.5)+H35)</f>
+        <f>SUM(D35+F35+(G35*5.5)+H35)</f>
         <v/>
       </c>
     </row>
@@ -2848,7 +2848,7 @@
       <c r="G36" s="227" t="n"/>
       <c r="H36" s="226" t="n"/>
       <c r="I36" s="228">
-        <f>SUM(F36+(G36*5.5)+H36)</f>
+        <f>SUM(D36+F36+(G36*5.5)+H36)</f>
         <v/>
       </c>
     </row>
@@ -2866,7 +2866,7 @@
       <c r="G37" s="231" t="n"/>
       <c r="H37" s="230" t="n"/>
       <c r="I37" s="232">
-        <f>SUM(F37+(G37*5.5)+H37)</f>
+        <f>SUM(D37+F37+(G37*5.5)+H37)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Expand quotation to 12 line items, fix R format and total formula
- Template expanded from 5 to 12 line item rows
- D column now shows R currency format
- TOTAL formula includes Skills Programme amount
- Frontend allows up to 12 line items
- Backend row references updated for new template layout

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Quotation Template.xlsx
+++ b/Quotation Template.xlsx
@@ -2147,7 +2147,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AA44"/>
+  <dimension ref="A1:AA51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" style="95" min="1" max="1"/>
@@ -2591,7 +2591,7 @@
       </c>
       <c r="B23" s="72" t="n"/>
       <c r="C23" s="78" t="n"/>
-      <c r="D23" s="186" t="n"/>
+      <c r="D23" s="79" t="n"/>
       <c r="E23" s="78" t="n"/>
       <c r="F23" s="186" t="n"/>
       <c r="G23" s="187" t="n"/>
@@ -2609,7 +2609,7 @@
       </c>
       <c r="B24" s="72" t="n"/>
       <c r="C24" s="78" t="n"/>
-      <c r="D24" s="186" t="n"/>
+      <c r="D24" s="79" t="n"/>
       <c r="E24" s="78" t="n"/>
       <c r="F24" s="186" t="n"/>
       <c r="G24" s="187" t="n"/>
@@ -2627,7 +2627,7 @@
       </c>
       <c r="B25" s="72" t="n"/>
       <c r="C25" s="78" t="n"/>
-      <c r="D25" s="186" t="n"/>
+      <c r="D25" s="79" t="n"/>
       <c r="E25" s="78" t="n"/>
       <c r="F25" s="186" t="n"/>
       <c r="G25" s="187" t="n"/>
@@ -2657,223 +2657,214 @@
       <c r="J26" s="189" t="n"/>
       <c r="K26" s="85" t="n"/>
     </row>
-    <row r="27" ht="14.45" customFormat="1" customHeight="1" s="84" thickBot="1">
-      <c r="A27" s="193" t="n"/>
-      <c r="B27" s="194" t="n"/>
-      <c r="C27" s="194" t="n"/>
-      <c r="D27" s="194" t="n"/>
-      <c r="E27" s="194" t="n"/>
-      <c r="F27" s="194" t="n"/>
-      <c r="G27" s="194" t="n"/>
-      <c r="H27" s="194" t="n"/>
-      <c r="I27" s="195" t="n"/>
+    <row r="27" customFormat="1" s="84">
+      <c r="A27" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B27" s="72" t="n"/>
+      <c r="C27" s="78" t="n"/>
+      <c r="D27" s="79" t="n"/>
+      <c r="E27" s="78" t="n"/>
+      <c r="F27" s="186" t="n"/>
+      <c r="G27" s="187" t="n"/>
+      <c r="H27" s="188" t="n"/>
+      <c r="I27" s="186">
+        <f>SUM(D27+F27+(G27*5.5)+H27)</f>
+        <v/>
+      </c>
+      <c r="J27" s="189" t="n"/>
       <c r="K27" s="85" t="n"/>
     </row>
-    <row r="28" hidden="1" ht="21.6" customFormat="1" customHeight="1" s="84">
-      <c r="A28" s="112" t="n">
+    <row r="28" customFormat="1" s="84">
+      <c r="A28" s="7" t="n">
+        <v>7</v>
+      </c>
+      <c r="B28" s="72" t="n"/>
+      <c r="C28" s="78" t="n"/>
+      <c r="D28" s="79" t="n"/>
+      <c r="E28" s="78" t="n"/>
+      <c r="F28" s="186" t="n"/>
+      <c r="G28" s="187" t="n"/>
+      <c r="H28" s="188" t="n"/>
+      <c r="I28" s="186">
+        <f>SUM(D28+F28+(G28*5.5)+H28)</f>
+        <v/>
+      </c>
+      <c r="J28" s="189" t="n"/>
+      <c r="K28" s="85" t="n"/>
+    </row>
+    <row r="29" customFormat="1" s="84">
+      <c r="A29" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="B29" s="72" t="n"/>
+      <c r="C29" s="78" t="n"/>
+      <c r="D29" s="79" t="n"/>
+      <c r="E29" s="78" t="n"/>
+      <c r="F29" s="186" t="n"/>
+      <c r="G29" s="187" t="n"/>
+      <c r="H29" s="188" t="n"/>
+      <c r="I29" s="186">
+        <f>SUM(D29+F29+(G29*5.5)+H29)</f>
+        <v/>
+      </c>
+      <c r="J29" s="189" t="n"/>
+      <c r="K29" s="85" t="n"/>
+    </row>
+    <row r="30" customFormat="1" s="84">
+      <c r="A30" s="7" t="n">
+        <v>9</v>
+      </c>
+      <c r="B30" s="72" t="n"/>
+      <c r="C30" s="78" t="n"/>
+      <c r="D30" s="79" t="n"/>
+      <c r="E30" s="78" t="n"/>
+      <c r="F30" s="186" t="n"/>
+      <c r="G30" s="187" t="n"/>
+      <c r="H30" s="188" t="n"/>
+      <c r="I30" s="186">
+        <f>SUM(D30+F30+(G30*5.5)+H30)</f>
+        <v/>
+      </c>
+      <c r="J30" s="189" t="n"/>
+      <c r="K30" s="85" t="n"/>
+    </row>
+    <row r="31" customFormat="1" s="84">
+      <c r="A31" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="B31" s="72" t="n"/>
+      <c r="C31" s="78" t="n"/>
+      <c r="D31" s="79" t="n"/>
+      <c r="E31" s="78" t="n"/>
+      <c r="F31" s="186" t="n"/>
+      <c r="G31" s="187" t="n"/>
+      <c r="H31" s="188" t="n"/>
+      <c r="I31" s="186">
+        <f>SUM(D31+F31+(G31*5.5)+H31)</f>
+        <v/>
+      </c>
+      <c r="J31" s="189" t="n"/>
+      <c r="K31" s="85" t="n"/>
+    </row>
+    <row r="32" customFormat="1" s="84">
+      <c r="A32" s="7" t="n">
+        <v>11</v>
+      </c>
+      <c r="B32" s="72" t="n"/>
+      <c r="C32" s="78" t="n"/>
+      <c r="D32" s="79" t="n"/>
+      <c r="E32" s="78" t="n"/>
+      <c r="F32" s="186" t="n"/>
+      <c r="G32" s="187" t="n"/>
+      <c r="H32" s="188" t="n"/>
+      <c r="I32" s="186">
+        <f>SUM(D32+F32+(G32*5.5)+H32)</f>
+        <v/>
+      </c>
+      <c r="J32" s="189" t="n"/>
+      <c r="K32" s="85" t="n"/>
+    </row>
+    <row r="33" customFormat="1" s="84">
+      <c r="A33" s="7" t="n">
+        <v>12</v>
+      </c>
+      <c r="B33" s="72" t="n"/>
+      <c r="C33" s="78" t="n"/>
+      <c r="D33" s="79" t="n"/>
+      <c r="E33" s="78" t="n"/>
+      <c r="F33" s="186" t="n"/>
+      <c r="G33" s="187" t="n"/>
+      <c r="H33" s="188" t="n"/>
+      <c r="I33" s="186">
+        <f>SUM(D33+F33+(G33*5.5)+H33)</f>
+        <v/>
+      </c>
+      <c r="J33" s="189" t="n"/>
+      <c r="K33" s="85" t="n"/>
+    </row>
+    <row r="34" ht="14.45" customFormat="1" customHeight="1" s="84" thickBot="1">
+      <c r="A34" s="193" t="n"/>
+      <c r="B34" s="194" t="n"/>
+      <c r="C34" s="194" t="n"/>
+      <c r="D34" s="194" t="n"/>
+      <c r="E34" s="194" t="n"/>
+      <c r="F34" s="194" t="n"/>
+      <c r="G34" s="194" t="n"/>
+      <c r="H34" s="194" t="n"/>
+      <c r="I34" s="195" t="n"/>
+      <c r="K34" s="85" t="n"/>
+    </row>
+    <row r="35" hidden="1" ht="21.6" customFormat="1" customHeight="1" s="84">
+      <c r="A35" s="112" t="n">
         <v>4</v>
       </c>
-      <c r="B28" s="196" t="inlineStr">
+      <c r="B35" s="196" t="inlineStr">
         <is>
           <t>Service cost (PAH,HAW)</t>
         </is>
       </c>
-      <c r="C28" s="197" t="n"/>
-      <c r="D28" s="198" t="n"/>
-      <c r="E28" s="199" t="n"/>
-      <c r="F28" s="117" t="n"/>
-      <c r="G28" s="118">
-        <f>F28&amp;"km"</f>
+      <c r="C35" s="197" t="n"/>
+      <c r="D35" s="198" t="n"/>
+      <c r="E35" s="199" t="n"/>
+      <c r="F35" s="117" t="n"/>
+      <c r="G35" s="118">
+        <f>F35&amp;"km"</f>
         <v/>
       </c>
-      <c r="H28" s="117" t="n"/>
-      <c r="I28" s="200">
-        <f>SUM(E28+(F28*5.5)+H28)</f>
+      <c r="H35" s="117" t="n"/>
+      <c r="I35" s="200">
+        <f>SUM(E35+(F35*5.5)+H35)</f>
         <v/>
       </c>
-      <c r="K28" s="85" t="n"/>
-    </row>
-    <row r="29" ht="20.45" customFormat="1" customHeight="1" s="84">
-      <c r="A29" s="124" t="n">
+      <c r="K35" s="85" t="n"/>
+    </row>
+    <row r="36" ht="20.45" customFormat="1" customHeight="1" s="84">
+      <c r="A36" s="124" t="n">
         <v>4</v>
       </c>
-      <c r="B29" s="201" t="inlineStr">
+      <c r="B36" s="201" t="inlineStr">
         <is>
           <t>Sampling</t>
         </is>
       </c>
-      <c r="C29" s="173" t="n"/>
-      <c r="D29" s="173" t="n"/>
-      <c r="E29" s="174" t="n"/>
-      <c r="F29" s="202" t="n"/>
-      <c r="G29" s="203" t="n"/>
-      <c r="H29" s="204" t="n"/>
-      <c r="I29" s="205">
-        <f>SUM(F29+(G29*5.5)+H29)</f>
+      <c r="C36" s="173" t="n"/>
+      <c r="D36" s="173" t="n"/>
+      <c r="E36" s="174" t="n"/>
+      <c r="F36" s="202" t="n"/>
+      <c r="G36" s="203" t="n"/>
+      <c r="H36" s="204" t="n"/>
+      <c r="I36" s="205">
+        <f>SUM(F36+(G36*5.5)+H36)</f>
         <v/>
       </c>
-      <c r="K29" s="85" t="n"/>
-    </row>
-    <row r="30" ht="19.35" customFormat="1" customHeight="1" s="84" thickBot="1">
-      <c r="A30" s="108" t="n">
+      <c r="K36" s="85" t="n"/>
+    </row>
+    <row r="37" ht="19.35" customFormat="1" customHeight="1" s="84" thickBot="1">
+      <c r="A37" s="108" t="n">
         <v>5</v>
       </c>
-      <c r="B30" s="206" t="inlineStr">
+      <c r="B37" s="206" t="inlineStr">
         <is>
           <t>Audit verification</t>
         </is>
       </c>
-      <c r="C30" s="180" t="n"/>
-      <c r="D30" s="180" t="n"/>
-      <c r="E30" s="181" t="n"/>
-      <c r="F30" s="207" t="n"/>
-      <c r="G30" s="208" t="n"/>
-      <c r="H30" s="209" t="n"/>
-      <c r="I30" s="210">
-        <f>SUM(F30+(G30*5.5)+H30)</f>
+      <c r="C37" s="180" t="n"/>
+      <c r="D37" s="180" t="n"/>
+      <c r="E37" s="181" t="n"/>
+      <c r="F37" s="207" t="n"/>
+      <c r="G37" s="208" t="n"/>
+      <c r="H37" s="209" t="n"/>
+      <c r="I37" s="210">
+        <f>SUM(F37+(G37*5.5)+H37)</f>
         <v/>
       </c>
-      <c r="K30" s="85" t="n"/>
-    </row>
-    <row r="31" ht="30" customFormat="1" customHeight="1" s="84" thickBot="1">
-      <c r="A31" s="211" t="inlineStr">
+      <c r="K37" s="85" t="n"/>
+    </row>
+    <row r="38" ht="30" customFormat="1" customHeight="1" s="84" thickBot="1">
+      <c r="A38" s="211" t="inlineStr">
         <is>
           <t>Sub - total</t>
-        </is>
-      </c>
-      <c r="B31" s="194" t="n"/>
-      <c r="C31" s="194" t="n"/>
-      <c r="D31" s="194" t="n"/>
-      <c r="E31" s="194" t="n"/>
-      <c r="F31" s="194" t="n"/>
-      <c r="G31" s="194" t="n"/>
-      <c r="H31" s="212" t="n"/>
-      <c r="I31" s="213">
-        <f>SUM(I22:I30)</f>
-        <v/>
-      </c>
-      <c r="K31" s="85" t="n"/>
-    </row>
-    <row r="32" hidden="1" ht="30" customFormat="1" customHeight="1" s="84">
-      <c r="A32" s="7" t="n"/>
-      <c r="B32" s="11" t="n"/>
-      <c r="C32" s="13" t="n"/>
-      <c r="D32" s="12" t="n"/>
-      <c r="E32" s="214" t="n"/>
-      <c r="F32" s="8" t="n"/>
-      <c r="G32" s="8" t="n"/>
-      <c r="H32" s="9" t="n"/>
-      <c r="I32" s="215" t="n"/>
-      <c r="K32" s="85" t="n"/>
-    </row>
-    <row r="33" hidden="1" ht="30" customFormat="1" customHeight="1" s="84">
-      <c r="A33" s="112" t="n"/>
-      <c r="B33" s="139" t="n"/>
-      <c r="C33" s="140" t="n"/>
-      <c r="D33" s="141" t="n"/>
-      <c r="E33" s="216" t="n"/>
-      <c r="F33" s="143" t="n"/>
-      <c r="G33" s="143" t="n"/>
-      <c r="H33" s="144" t="n"/>
-      <c r="I33" s="217" t="n"/>
-      <c r="K33" s="85" t="n"/>
-    </row>
-    <row r="34" ht="16.5" customFormat="1" customHeight="1" s="218">
-      <c r="A34" s="242" t="inlineStr">
-        <is>
-          <t>Conducting an audit verification &amp; sampling enables us to provide you with a discount.</t>
-        </is>
-      </c>
-      <c r="B34" s="170" t="n"/>
-      <c r="C34" s="220" t="inlineStr">
-        <is>
-          <t>Discounted</t>
-        </is>
-      </c>
-      <c r="D34" s="220" t="n"/>
-      <c r="E34" s="174" t="n"/>
-      <c r="F34" s="221" t="n"/>
-      <c r="G34" s="222" t="n"/>
-      <c r="H34" s="223" t="n"/>
-      <c r="I34" s="224">
-        <f>SUM(D34+F34+(G34*5.5)+H34)</f>
-        <v/>
-      </c>
-      <c r="J34" s="189" t="n"/>
-      <c r="K34" s="189" t="n"/>
-      <c r="L34" s="189" t="n"/>
-      <c r="M34" s="189" t="n"/>
-      <c r="N34" s="189" t="n"/>
-      <c r="O34" s="189" t="n"/>
-      <c r="P34" s="189" t="n"/>
-      <c r="Q34" s="189" t="n"/>
-      <c r="R34" s="189" t="n"/>
-      <c r="S34" s="189" t="n"/>
-      <c r="T34" s="189" t="n"/>
-      <c r="U34" s="189" t="n"/>
-      <c r="V34" s="189" t="n"/>
-      <c r="W34" s="189" t="n"/>
-      <c r="X34" s="189" t="n"/>
-      <c r="Y34" s="189" t="n"/>
-      <c r="Z34" s="189" t="n"/>
-      <c r="AA34" s="189" t="n"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="22" t="n"/>
-      <c r="C35" s="225" t="inlineStr">
-        <is>
-          <t>Discounted</t>
-        </is>
-      </c>
-      <c r="D35" s="225" t="n"/>
-      <c r="E35" s="176" t="n"/>
-      <c r="F35" s="226" t="n"/>
-      <c r="G35" s="227" t="n"/>
-      <c r="H35" s="226" t="n"/>
-      <c r="I35" s="228">
-        <f>SUM(D35+F35+(G35*5.5)+H35)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="22" t="n"/>
-      <c r="C36" s="225" t="inlineStr">
-        <is>
-          <t>Discounted</t>
-        </is>
-      </c>
-      <c r="D36" s="225" t="n"/>
-      <c r="E36" s="176" t="n"/>
-      <c r="F36" s="226" t="n"/>
-      <c r="G36" s="227" t="n"/>
-      <c r="H36" s="226" t="n"/>
-      <c r="I36" s="228">
-        <f>SUM(D36+F36+(G36*5.5)+H36)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="37" ht="15.75" customHeight="1" s="95" thickBot="1">
-      <c r="A37" s="23" t="n"/>
-      <c r="B37" s="1" t="n"/>
-      <c r="C37" s="229" t="inlineStr">
-        <is>
-          <t>Discounted</t>
-        </is>
-      </c>
-      <c r="D37" s="229" t="n"/>
-      <c r="E37" s="181" t="n"/>
-      <c r="F37" s="230" t="n"/>
-      <c r="G37" s="231" t="n"/>
-      <c r="H37" s="230" t="n"/>
-      <c r="I37" s="232">
-        <f>SUM(D37+F37+(G37*5.5)+H37)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="38" ht="22.5" customFormat="1" customHeight="1" s="5">
-      <c r="A38" s="233" t="inlineStr">
-        <is>
-          <t>Discount provided</t>
         </is>
       </c>
       <c r="B38" s="194" t="n"/>
@@ -2883,115 +2874,250 @@
       <c r="F38" s="194" t="n"/>
       <c r="G38" s="194" t="n"/>
       <c r="H38" s="212" t="n"/>
-      <c r="I38" s="234">
-        <f>SUM(I34:I37)</f>
+      <c r="I38" s="213">
+        <f>SUM(I22:I37)</f>
         <v/>
       </c>
-    </row>
-    <row r="39" ht="19.5" customFormat="1" customHeight="1" s="5" thickBot="1">
-      <c r="A39" s="235" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> TOTAL Excl 15% VAT</t>
-        </is>
-      </c>
-      <c r="B39" s="180" t="n"/>
-      <c r="C39" s="180" t="n"/>
-      <c r="D39" s="180" t="n"/>
-      <c r="E39" s="180" t="n"/>
-      <c r="F39" s="180" t="n"/>
-      <c r="G39" s="180" t="n"/>
-      <c r="H39" s="236" t="n"/>
-      <c r="I39" s="237">
-        <f>I31+I38</f>
+      <c r="K38" s="85" t="n"/>
+    </row>
+    <row r="39" hidden="1" ht="30" customFormat="1" customHeight="1" s="84">
+      <c r="A39" s="7" t="n"/>
+      <c r="B39" s="11" t="n"/>
+      <c r="C39" s="13" t="n"/>
+      <c r="D39" s="12" t="n"/>
+      <c r="E39" s="214" t="n"/>
+      <c r="F39" s="8" t="n"/>
+      <c r="G39" s="8" t="n"/>
+      <c r="H39" s="9" t="n"/>
+      <c r="I39" s="215" t="n"/>
+      <c r="K39" s="85" t="n"/>
+    </row>
+    <row r="40" hidden="1" ht="30" customFormat="1" customHeight="1" s="84">
+      <c r="A40" s="112" t="n"/>
+      <c r="B40" s="139" t="n"/>
+      <c r="C40" s="140" t="n"/>
+      <c r="D40" s="141" t="n"/>
+      <c r="E40" s="216" t="n"/>
+      <c r="F40" s="143" t="n"/>
+      <c r="G40" s="143" t="n"/>
+      <c r="H40" s="144" t="n"/>
+      <c r="I40" s="217" t="n"/>
+      <c r="K40" s="85" t="n"/>
+    </row>
+    <row r="41" ht="16.5" customFormat="1" customHeight="1" s="218">
+      <c r="A41" s="242" t="inlineStr">
+        <is>
+          <t>Conducting an audit verification &amp; sampling enables us to provide you with a discount.</t>
+        </is>
+      </c>
+      <c r="B41" s="170" t="n"/>
+      <c r="C41" s="220" t="inlineStr">
+        <is>
+          <t>Discounted</t>
+        </is>
+      </c>
+      <c r="D41" s="220" t="n"/>
+      <c r="E41" s="174" t="n"/>
+      <c r="F41" s="221" t="n"/>
+      <c r="G41" s="222" t="n"/>
+      <c r="H41" s="223" t="n"/>
+      <c r="I41" s="224">
+        <f>SUM(F41+(G41*5.5)+H41)</f>
         <v/>
       </c>
-    </row>
-    <row r="40" ht="23.45" customHeight="1" s="95">
-      <c r="A40" s="238" t="inlineStr">
-        <is>
-          <t>For acceptance of the quote, please sign below and email back the signed copy</t>
-        </is>
-      </c>
-      <c r="B40" s="170" t="n"/>
-      <c r="C40" s="170" t="n"/>
-      <c r="D40" s="170" t="n"/>
-      <c r="E40" s="170" t="n"/>
-      <c r="F40" s="170" t="n"/>
-      <c r="G40" s="170" t="n"/>
-      <c r="H40" s="170" t="n"/>
-      <c r="I40" s="239" t="n"/>
-    </row>
-    <row r="41" ht="26.1" customHeight="1" s="95">
-      <c r="A41" s="22" t="n"/>
-      <c r="B41" s="70" t="n"/>
-      <c r="C41" s="194" t="n"/>
-      <c r="E41" s="168" t="n"/>
-      <c r="H41" s="71" t="n"/>
-      <c r="I41" s="195" t="n"/>
+      <c r="J41" s="189" t="n"/>
+      <c r="K41" s="189" t="n"/>
+      <c r="L41" s="189" t="n"/>
+      <c r="M41" s="189" t="n"/>
+      <c r="N41" s="189" t="n"/>
+      <c r="O41" s="189" t="n"/>
+      <c r="P41" s="189" t="n"/>
+      <c r="Q41" s="189" t="n"/>
+      <c r="R41" s="189" t="n"/>
+      <c r="S41" s="189" t="n"/>
+      <c r="T41" s="189" t="n"/>
+      <c r="U41" s="189" t="n"/>
+      <c r="V41" s="189" t="n"/>
+      <c r="W41" s="189" t="n"/>
+      <c r="X41" s="189" t="n"/>
+      <c r="Y41" s="189" t="n"/>
+      <c r="Z41" s="189" t="n"/>
+      <c r="AA41" s="189" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="22" t="n"/>
-      <c r="B42" s="97" t="inlineStr">
+      <c r="C42" s="225" t="inlineStr">
+        <is>
+          <t>Discounted</t>
+        </is>
+      </c>
+      <c r="D42" s="225" t="n"/>
+      <c r="E42" s="176" t="n"/>
+      <c r="F42" s="226" t="n"/>
+      <c r="G42" s="227" t="n"/>
+      <c r="H42" s="226" t="n"/>
+      <c r="I42" s="228">
+        <f>SUM(F42+(G42*5.5)+H42)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="22" t="n"/>
+      <c r="C43" s="225" t="inlineStr">
+        <is>
+          <t>Discounted</t>
+        </is>
+      </c>
+      <c r="D43" s="225" t="n"/>
+      <c r="E43" s="176" t="n"/>
+      <c r="F43" s="226" t="n"/>
+      <c r="G43" s="227" t="n"/>
+      <c r="H43" s="226" t="n"/>
+      <c r="I43" s="228">
+        <f>SUM(F43+(G43*5.5)+H43)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44" ht="15.75" customHeight="1" s="95" thickBot="1">
+      <c r="A44" s="23" t="n"/>
+      <c r="B44" s="1" t="n"/>
+      <c r="C44" s="229" t="inlineStr">
+        <is>
+          <t>Discounted</t>
+        </is>
+      </c>
+      <c r="D44" s="229" t="n"/>
+      <c r="E44" s="181" t="n"/>
+      <c r="F44" s="230" t="n"/>
+      <c r="G44" s="231" t="n"/>
+      <c r="H44" s="230" t="n"/>
+      <c r="I44" s="232">
+        <f>SUM(F44+(G44*5.5)+H44)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45" ht="22.5" customFormat="1" customHeight="1" s="5">
+      <c r="A45" s="233" t="inlineStr">
+        <is>
+          <t>Discount provided</t>
+        </is>
+      </c>
+      <c r="B45" s="194" t="n"/>
+      <c r="C45" s="194" t="n"/>
+      <c r="D45" s="194" t="n"/>
+      <c r="E45" s="194" t="n"/>
+      <c r="F45" s="194" t="n"/>
+      <c r="G45" s="194" t="n"/>
+      <c r="H45" s="212" t="n"/>
+      <c r="I45" s="234">
+        <f>SUM(I41:I44)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46" ht="19.5" customFormat="1" customHeight="1" s="5" thickBot="1">
+      <c r="A46" s="235" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> TOTAL Excl 15% VAT</t>
+        </is>
+      </c>
+      <c r="B46" s="180" t="n"/>
+      <c r="C46" s="180" t="n"/>
+      <c r="D46" s="180" t="n"/>
+      <c r="E46" s="180" t="n"/>
+      <c r="F46" s="180" t="n"/>
+      <c r="G46" s="180" t="n"/>
+      <c r="H46" s="236" t="n"/>
+      <c r="I46" s="237">
+        <f>I38+I45</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47" ht="23.45" customHeight="1" s="95">
+      <c r="A47" s="238" t="inlineStr">
+        <is>
+          <t>For acceptance of the quote, please sign below and email back the signed copy</t>
+        </is>
+      </c>
+      <c r="B47" s="170" t="n"/>
+      <c r="C47" s="170" t="n"/>
+      <c r="D47" s="170" t="n"/>
+      <c r="E47" s="170" t="n"/>
+      <c r="F47" s="170" t="n"/>
+      <c r="G47" s="170" t="n"/>
+      <c r="H47" s="170" t="n"/>
+      <c r="I47" s="239" t="n"/>
+    </row>
+    <row r="48" ht="26.1" customHeight="1" s="95">
+      <c r="A48" s="22" t="n"/>
+      <c r="B48" s="70" t="n"/>
+      <c r="C48" s="194" t="n"/>
+      <c r="E48" s="168" t="n"/>
+      <c r="H48" s="71" t="n"/>
+      <c r="I48" s="195" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="22" t="n"/>
+      <c r="B49" s="97" t="inlineStr">
         <is>
           <t>Client</t>
         </is>
       </c>
-      <c r="C42" s="97" t="n"/>
-      <c r="E42" s="168" t="n"/>
-      <c r="H42" s="69" t="inlineStr">
+      <c r="C49" s="97" t="n"/>
+      <c r="E49" s="168" t="n"/>
+      <c r="H49" s="69" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="I42" s="240" t="n"/>
-    </row>
-    <row r="43" ht="15.75" customHeight="1" s="95" thickBot="1">
-      <c r="A43" s="23" t="n"/>
-      <c r="B43" s="1" t="n"/>
-      <c r="C43" s="1" t="n"/>
-      <c r="D43" s="1" t="n"/>
-      <c r="E43" s="169" t="n"/>
-      <c r="F43" s="1" t="n"/>
-      <c r="G43" s="1" t="n"/>
-      <c r="H43" s="1" t="n"/>
-      <c r="I43" s="241" t="n"/>
-    </row>
-    <row r="44" ht="52.5" customHeight="1" s="95">
-      <c r="A44" s="67" t="inlineStr">
+      <c r="I49" s="240" t="n"/>
+    </row>
+    <row r="50" ht="15.75" customHeight="1" s="95" thickBot="1">
+      <c r="A50" s="23" t="n"/>
+      <c r="B50" s="1" t="n"/>
+      <c r="C50" s="1" t="n"/>
+      <c r="D50" s="1" t="n"/>
+      <c r="E50" s="169" t="n"/>
+      <c r="F50" s="1" t="n"/>
+      <c r="G50" s="1" t="n"/>
+      <c r="H50" s="1" t="n"/>
+      <c r="I50" s="241" t="n"/>
+    </row>
+    <row r="51" ht="52.5" customHeight="1" s="95">
+      <c r="A51" s="67" t="inlineStr">
         <is>
           <t xml:space="preserve">General Manager : Dr GC Neethling
  Red Meat Abattoir Association                                                                     Abattoir Skills Training
 </t>
         </is>
       </c>
-      <c r="B44" s="170" t="n"/>
-      <c r="C44" s="170" t="n"/>
-      <c r="D44" s="170" t="n"/>
-      <c r="E44" s="170" t="n"/>
-      <c r="F44" s="170" t="n"/>
-      <c r="G44" s="170" t="n"/>
-      <c r="H44" s="170" t="n"/>
-      <c r="I44" s="170" t="n"/>
+      <c r="B51" s="170" t="n"/>
+      <c r="C51" s="170" t="n"/>
+      <c r="D51" s="170" t="n"/>
+      <c r="E51" s="170" t="n"/>
+      <c r="F51" s="170" t="n"/>
+      <c r="G51" s="170" t="n"/>
+      <c r="H51" s="170" t="n"/>
+      <c r="I51" s="170" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="55">
     <mergeCell ref="D11:I11"/>
     <mergeCell ref="D2:I2"/>
-    <mergeCell ref="A39:H39"/>
+    <mergeCell ref="A46:H46"/>
     <mergeCell ref="D13:I13"/>
-    <mergeCell ref="D34:E34"/>
-    <mergeCell ref="B30:E30"/>
+    <mergeCell ref="D41:E41"/>
+    <mergeCell ref="B37:E37"/>
     <mergeCell ref="D17:I17"/>
     <mergeCell ref="A18:C18"/>
-    <mergeCell ref="H41:I41"/>
-    <mergeCell ref="A27:I27"/>
+    <mergeCell ref="H48:I48"/>
+    <mergeCell ref="A34:I34"/>
     <mergeCell ref="A3:C3"/>
     <mergeCell ref="A12:C12"/>
     <mergeCell ref="D16:I16"/>
-    <mergeCell ref="D36:E36"/>
+    <mergeCell ref="D43:E43"/>
     <mergeCell ref="D7:I7"/>
     <mergeCell ref="A2:C2"/>
-    <mergeCell ref="B28:D28"/>
+    <mergeCell ref="B35:D35"/>
     <mergeCell ref="A5:C5"/>
     <mergeCell ref="D4:I4"/>
     <mergeCell ref="A14:C14"/>
@@ -3009,27 +3135,27 @@
     <mergeCell ref="A21:B21"/>
     <mergeCell ref="A13:C13"/>
     <mergeCell ref="A19:C19"/>
-    <mergeCell ref="A34:B37"/>
+    <mergeCell ref="A41:B44"/>
     <mergeCell ref="D14:I14"/>
     <mergeCell ref="D5:I5"/>
-    <mergeCell ref="A44:I44"/>
-    <mergeCell ref="D37:E37"/>
-    <mergeCell ref="A40:I40"/>
+    <mergeCell ref="A51:I51"/>
+    <mergeCell ref="D44:E44"/>
+    <mergeCell ref="A47:I47"/>
     <mergeCell ref="A9:C9"/>
     <mergeCell ref="A15:C15"/>
     <mergeCell ref="D19:I19"/>
     <mergeCell ref="D10:I10"/>
     <mergeCell ref="A11:C11"/>
+    <mergeCell ref="A45:H45"/>
+    <mergeCell ref="H49:I49"/>
+    <mergeCell ref="A6:C6"/>
+    <mergeCell ref="B36:E36"/>
+    <mergeCell ref="D6:I6"/>
+    <mergeCell ref="B48:C48"/>
+    <mergeCell ref="A7:C7"/>
     <mergeCell ref="A38:H38"/>
-    <mergeCell ref="H42:I42"/>
-    <mergeCell ref="A6:C6"/>
-    <mergeCell ref="B29:E29"/>
-    <mergeCell ref="D6:I6"/>
-    <mergeCell ref="B41:C41"/>
-    <mergeCell ref="A7:C7"/>
-    <mergeCell ref="A31:H31"/>
     <mergeCell ref="A16:C16"/>
-    <mergeCell ref="D35:E35"/>
+    <mergeCell ref="D42:E42"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D13" r:id="rId1"/>

</xml_diff>

<commit_message>
Fix quotation logo: remove transparency effect, resize to proper dimensions
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Quotation Template.xlsx
+++ b/Quotation Template.xlsx
@@ -1692,12 +1692,7 @@
         </cNvPicPr>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1">
-          <clrChange>
-            <clrFrom/>
-            <clrTo/>
-          </clrChange>
-        </a:blip>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
         <a:srcRect xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
@@ -1744,12 +1739,7 @@
         </cNvPicPr>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2">
-          <clrChange>
-            <clrFrom/>
-            <clrTo/>
-          </clrChange>
-        </a:blip>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
         <a:srcRect xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>

</xml_diff>

<commit_message>
Fix bottom logo positions: shift drawing anchors to row 50 after template expansion
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Quotation Template.xlsx
+++ b/Quotation Template.xlsx
@@ -1675,13 +1675,13 @@
     <from>
       <col>0</col>
       <colOff>97291</colOff>
-      <row>43</row>
+      <row>50</row>
       <rowOff>46377</rowOff>
     </from>
     <to>
       <col>1</col>
       <colOff>297656</colOff>
-      <row>43</row>
+      <row>50</row>
       <rowOff>639103</rowOff>
     </to>
     <pic>
@@ -1806,13 +1806,13 @@
     <from>
       <col>8</col>
       <colOff>98880</colOff>
-      <row>43</row>
+      <row>50</row>
       <rowOff>32945</rowOff>
     </from>
     <to>
       <col>9</col>
       <colOff>2211</colOff>
-      <row>43</row>
+      <row>50</row>
       <rowOff>659475</rowOff>
     </to>
     <pic>

</xml_diff>

<commit_message>
Fix quotation: remove bold separator, label Sampling/Audit as A/B, hide blank rows
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Quotation Template.xlsx
+++ b/Quotation Template.xlsx
@@ -2773,7 +2773,7 @@
       <c r="J33" s="189" t="n"/>
       <c r="K33" s="85" t="n"/>
     </row>
-    <row r="34" ht="14.45" customFormat="1" customHeight="1" s="84" thickBot="1">
+    <row r="34" ht="14.45" customFormat="1" customHeight="1" s="84">
       <c r="A34" s="193" t="n"/>
       <c r="B34" s="194" t="n"/>
       <c r="C34" s="194" t="n"/>
@@ -2810,8 +2810,10 @@
       <c r="K35" s="85" t="n"/>
     </row>
     <row r="36" ht="20.45" customFormat="1" customHeight="1" s="84">
-      <c r="A36" s="124" t="n">
-        <v>4</v>
+      <c r="A36" s="124" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
       </c>
       <c r="B36" s="201" t="inlineStr">
         <is>
@@ -2831,8 +2833,10 @@
       <c r="K36" s="85" t="n"/>
     </row>
     <row r="37" ht="19.35" customFormat="1" customHeight="1" s="84" thickBot="1">
-      <c r="A37" s="108" t="n">
-        <v>5</v>
+      <c r="A37" s="108" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
       </c>
       <c r="B37" s="206" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Fix quotation template: Rand format for all Skills Programme amounts, centre discount accommodation
Rows 23-33 of the Skills Programme Amount column had General format
(only rows 22 and 26 showed Rand values). The Skills Programme discount
accommodation cell (H41) was left-aligned and bold, unlike the rest of
the discount grid.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Quotation Template.xlsx
+++ b/Quotation Template.xlsx
@@ -996,7 +996,7 @@
     </xf>
     <xf numFmtId="169" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="243">
+  <cellXfs count="245">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1656,6 +1656,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="23" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="22" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="30" fillId="0" borderId="50" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf applyNumberFormat="1" numFmtId="164" fontId="6" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="28" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2581,7 +2587,7 @@
       </c>
       <c r="B23" s="72" t="n"/>
       <c r="C23" s="78" t="n"/>
-      <c r="D23" s="79" t="n"/>
+      <c r="D23" s="243" t="n"/>
       <c r="E23" s="78" t="n"/>
       <c r="F23" s="186" t="n"/>
       <c r="G23" s="187" t="n"/>
@@ -2599,7 +2605,7 @@
       </c>
       <c r="B24" s="72" t="n"/>
       <c r="C24" s="78" t="n"/>
-      <c r="D24" s="79" t="n"/>
+      <c r="D24" s="243" t="n"/>
       <c r="E24" s="78" t="n"/>
       <c r="F24" s="186" t="n"/>
       <c r="G24" s="187" t="n"/>
@@ -2617,7 +2623,7 @@
       </c>
       <c r="B25" s="72" t="n"/>
       <c r="C25" s="78" t="n"/>
-      <c r="D25" s="79" t="n"/>
+      <c r="D25" s="243" t="n"/>
       <c r="E25" s="78" t="n"/>
       <c r="F25" s="186" t="n"/>
       <c r="G25" s="187" t="n"/>
@@ -2653,7 +2659,7 @@
       </c>
       <c r="B27" s="72" t="n"/>
       <c r="C27" s="78" t="n"/>
-      <c r="D27" s="79" t="n"/>
+      <c r="D27" s="243" t="n"/>
       <c r="E27" s="78" t="n"/>
       <c r="F27" s="186" t="n"/>
       <c r="G27" s="187" t="n"/>
@@ -2671,7 +2677,7 @@
       </c>
       <c r="B28" s="72" t="n"/>
       <c r="C28" s="78" t="n"/>
-      <c r="D28" s="79" t="n"/>
+      <c r="D28" s="243" t="n"/>
       <c r="E28" s="78" t="n"/>
       <c r="F28" s="186" t="n"/>
       <c r="G28" s="187" t="n"/>
@@ -2689,7 +2695,7 @@
       </c>
       <c r="B29" s="72" t="n"/>
       <c r="C29" s="78" t="n"/>
-      <c r="D29" s="79" t="n"/>
+      <c r="D29" s="243" t="n"/>
       <c r="E29" s="78" t="n"/>
       <c r="F29" s="186" t="n"/>
       <c r="G29" s="187" t="n"/>
@@ -2707,7 +2713,7 @@
       </c>
       <c r="B30" s="72" t="n"/>
       <c r="C30" s="78" t="n"/>
-      <c r="D30" s="79" t="n"/>
+      <c r="D30" s="243" t="n"/>
       <c r="E30" s="78" t="n"/>
       <c r="F30" s="186" t="n"/>
       <c r="G30" s="187" t="n"/>
@@ -2725,7 +2731,7 @@
       </c>
       <c r="B31" s="72" t="n"/>
       <c r="C31" s="78" t="n"/>
-      <c r="D31" s="79" t="n"/>
+      <c r="D31" s="243" t="n"/>
       <c r="E31" s="78" t="n"/>
       <c r="F31" s="186" t="n"/>
       <c r="G31" s="187" t="n"/>
@@ -2743,7 +2749,7 @@
       </c>
       <c r="B32" s="72" t="n"/>
       <c r="C32" s="78" t="n"/>
-      <c r="D32" s="79" t="n"/>
+      <c r="D32" s="243" t="n"/>
       <c r="E32" s="78" t="n"/>
       <c r="F32" s="186" t="n"/>
       <c r="G32" s="187" t="n"/>
@@ -2761,7 +2767,7 @@
       </c>
       <c r="B33" s="72" t="n"/>
       <c r="C33" s="78" t="n"/>
-      <c r="D33" s="79" t="n"/>
+      <c r="D33" s="243" t="n"/>
       <c r="E33" s="78" t="n"/>
       <c r="F33" s="186" t="n"/>
       <c r="G33" s="187" t="n"/>
@@ -2914,7 +2920,7 @@
       <c r="E41" s="174" t="n"/>
       <c r="F41" s="221" t="n"/>
       <c r="G41" s="222" t="n"/>
-      <c r="H41" s="223" t="n"/>
+      <c r="H41" s="221" t="n"/>
       <c r="I41" s="224">
         <f>SUM(F41+(G41*5.5)+H41)</f>
         <v/>

</xml_diff>